<commit_message>
fix(migration): vendor-accurate fixtures, honest CCH guidance, Step 4 client preview
- fixtures: EF Status columns use real e-file ACK statuses (Drake/ProSeries);
  status vs notes carry distinct realistic per-vendor values; 1041 trust
  deadline corrected to 09/30; regenerate all realistic-exports fixtures
- intake: reword CCH .rtnbak/.rctrl guidance to cover Axcess + ProSystem fx
  (+ zh-CN); fix README .dif/.fbk stub wording
- dry-run: add per-client preview (clientsPreview on DryRunSummary) so Step 4
  confirms by outcome instead of by column schema

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product-design/migration-copilot/06-fixtures/realistic-exports/karbon-all-contacts.xlsx
+++ b/docs/product-design/migration-copilot/06-fixtures/realistic-exports/karbon-all-contacts.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="215">
   <si>
     <t>ContactKey</t>
   </si>
@@ -76,7 +76,7 @@
     <t>CA</t>
   </si>
   <si>
-    <t>1065; In Progress</t>
+    <t>1065; Ready for Review</t>
   </si>
   <si>
     <t>In Progress</t>
@@ -106,7 +106,7 @@
     <t>NY</t>
   </si>
   <si>
-    <t>1065; Waiting on client</t>
+    <t>1065; On Extension</t>
   </si>
   <si>
     <t>Waiting on client</t>
@@ -136,7 +136,7 @@
     <t>TX</t>
   </si>
   <si>
-    <t>1120; Ready for review</t>
+    <t>1120; Waiting on Client</t>
   </si>
   <si>
     <t>Ready for review</t>
@@ -169,7 +169,7 @@
     <t>FL</t>
   </si>
   <si>
-    <t>1040; Organizer sent</t>
+    <t>1040; Complete</t>
   </si>
   <si>
     <t>Organizer sent</t>
@@ -196,7 +196,7 @@
     <t>WA</t>
   </si>
   <si>
-    <t>1065; Open items</t>
+    <t>1065; Not Started</t>
   </si>
   <si>
     <t>Open items</t>
@@ -223,7 +223,7 @@
     <t>IL</t>
   </si>
   <si>
-    <t>1041; Extension filed</t>
+    <t>1041; In Progress</t>
   </si>
   <si>
     <t>Extension filed</t>
@@ -247,7 +247,7 @@
     <t>99-1000007</t>
   </si>
   <si>
-    <t>Schedule C; Needs bookkeeping</t>
+    <t>Schedule C; Ready for Review</t>
   </si>
   <si>
     <t>Needs bookkeeping</t>
@@ -271,7 +271,7 @@
     <t>99-1000008</t>
   </si>
   <si>
-    <t>990; Board review</t>
+    <t>990; On Extension</t>
   </si>
   <si>
     <t>Board review</t>
@@ -295,7 +295,7 @@
     <t>99-1000009</t>
   </si>
   <si>
-    <t>1065; In progress</t>
+    <t>1065; Waiting on Client</t>
   </si>
   <si>
     <t>In progress</t>
@@ -319,7 +319,7 @@
     <t>99-1000010</t>
   </si>
   <si>
-    <t>1120S; Ready for e-file</t>
+    <t>1120S; Complete</t>
   </si>
   <si>
     <t>Ready for e-file</t>
@@ -343,7 +343,7 @@
     <t>99-1000011</t>
   </si>
   <si>
-    <t>1120; R&amp;D credit review</t>
+    <t>1120; Not Started</t>
   </si>
   <si>
     <t>R&amp;D credit review</t>
@@ -367,7 +367,7 @@
     <t>99-1000012</t>
   </si>
   <si>
-    <t>1040; Missing K-1</t>
+    <t>1040; In Progress</t>
   </si>
   <si>
     <t>Missing K-1</t>
@@ -391,9 +391,6 @@
     <t>99-1000013</t>
   </si>
   <si>
-    <t>1065; Partner capital review</t>
-  </si>
-  <si>
     <t>Partner capital review</t>
   </si>
   <si>
@@ -415,7 +412,7 @@
     <t>99-1000014</t>
   </si>
   <si>
-    <t>1041; Beneficiary update</t>
+    <t>1041; On Extension</t>
   </si>
   <si>
     <t>Beneficiary update</t>
@@ -439,7 +436,7 @@
     <t>99-1000015</t>
   </si>
   <si>
-    <t>Schedule C; Mileage log pending</t>
+    <t>Schedule C; Waiting on Client</t>
   </si>
   <si>
     <t>Mileage log pending</t>
@@ -463,7 +460,7 @@
     <t>99-1000016</t>
   </si>
   <si>
-    <t>1065; Multi-member LLC</t>
+    <t>1065; Complete</t>
   </si>
   <si>
     <t>Multi-member LLC</t>
@@ -487,7 +484,7 @@
     <t>99-1000017</t>
   </si>
   <si>
-    <t>1120S; Payroll tie-out</t>
+    <t>1120S; Not Started</t>
   </si>
   <si>
     <t>Payroll tie-out</t>
@@ -511,7 +508,7 @@
     <t>99-1000018</t>
   </si>
   <si>
-    <t>1120; Inventory review</t>
+    <t>1120; In Progress</t>
   </si>
   <si>
     <t>Inventory review</t>
@@ -538,9 +535,6 @@
     <t/>
   </si>
   <si>
-    <t>1065; Review: missing filing state</t>
-  </si>
-  <si>
     <t>Review: missing filing state</t>
   </si>
   <si>
@@ -565,7 +559,7 @@
     <t>C.A.</t>
   </si>
   <si>
-    <t>1120S; Review: state exported as C.A.</t>
+    <t>1120S; On Extension</t>
   </si>
   <si>
     <t>Review: state exported as C.A.</t>
@@ -589,9 +583,6 @@
     <t>99-1000021</t>
   </si>
   <si>
-    <t>1065; Owner basis review</t>
-  </si>
-  <si>
     <t>Owner basis review</t>
   </si>
   <si>
@@ -613,9 +604,6 @@
     <t>99-1000022</t>
   </si>
   <si>
-    <t>1040; Schedule E rental</t>
-  </si>
-  <si>
     <t>Schedule E rental</t>
   </si>
   <si>
@@ -637,7 +625,7 @@
     <t>99-1000023</t>
   </si>
   <si>
-    <t>1041; Estimated tax review</t>
+    <t>1041; Not Started</t>
   </si>
   <si>
     <t>Estimated tax review</t>
@@ -661,7 +649,7 @@
     <t>99-1000024</t>
   </si>
   <si>
-    <t>990; Grant schedule review</t>
+    <t>990; In Progress</t>
   </si>
   <si>
     <t>Grant schedule review</t>
@@ -1199,27 +1187,27 @@
         <v>21</v>
       </c>
       <c r="K14" t="s">
+        <v>22</v>
+      </c>
+      <c r="L14" t="s">
         <v>127</v>
-      </c>
-      <c r="L14" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
+        <v>128</v>
+      </c>
+      <c r="B15" t="s">
         <v>129</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>130</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>131</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>132</v>
-      </c>
-      <c r="E15" t="s">
-        <v>133</v>
       </c>
       <c r="F15" t="s">
         <v>29</v>
@@ -1228,7 +1216,7 @@
         <v>18</v>
       </c>
       <c r="H15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I15" t="s">
         <v>20</v>
@@ -1237,27 +1225,27 @@
         <v>31</v>
       </c>
       <c r="K15" t="s">
+        <v>134</v>
+      </c>
+      <c r="L15" t="s">
         <v>135</v>
-      </c>
-      <c r="L15" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
+        <v>136</v>
+      </c>
+      <c r="B16" t="s">
         <v>137</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>138</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>139</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>140</v>
-      </c>
-      <c r="E16" t="s">
-        <v>141</v>
       </c>
       <c r="F16" t="s">
         <v>39</v>
@@ -1266,7 +1254,7 @@
         <v>18</v>
       </c>
       <c r="H16" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I16" t="s">
         <v>20</v>
@@ -1275,27 +1263,27 @@
         <v>41</v>
       </c>
       <c r="K16" t="s">
+        <v>142</v>
+      </c>
+      <c r="L16" t="s">
         <v>143</v>
-      </c>
-      <c r="L16" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
+        <v>144</v>
+      </c>
+      <c r="B17" t="s">
         <v>145</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>146</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>147</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>148</v>
-      </c>
-      <c r="E17" t="s">
-        <v>149</v>
       </c>
       <c r="F17" t="s">
         <v>49</v>
@@ -1304,7 +1292,7 @@
         <v>18</v>
       </c>
       <c r="H17" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I17" t="s">
         <v>20</v>
@@ -1313,27 +1301,27 @@
         <v>52</v>
       </c>
       <c r="K17" t="s">
+        <v>150</v>
+      </c>
+      <c r="L17" t="s">
         <v>151</v>
-      </c>
-      <c r="L17" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
+        <v>152</v>
+      </c>
+      <c r="B18" t="s">
         <v>153</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>154</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>155</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>156</v>
-      </c>
-      <c r="E18" t="s">
-        <v>157</v>
       </c>
       <c r="F18" t="s">
         <v>17</v>
@@ -1342,7 +1330,7 @@
         <v>18</v>
       </c>
       <c r="H18" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I18" t="s">
         <v>20</v>
@@ -1351,27 +1339,27 @@
         <v>61</v>
       </c>
       <c r="K18" t="s">
+        <v>158</v>
+      </c>
+      <c r="L18" t="s">
         <v>159</v>
-      </c>
-      <c r="L18" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
+        <v>160</v>
+      </c>
+      <c r="B19" t="s">
         <v>161</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>162</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>163</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>164</v>
-      </c>
-      <c r="E19" t="s">
-        <v>165</v>
       </c>
       <c r="F19" t="s">
         <v>29</v>
@@ -1380,7 +1368,7 @@
         <v>18</v>
       </c>
       <c r="H19" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I19" t="s">
         <v>20</v>
@@ -1389,27 +1377,27 @@
         <v>70</v>
       </c>
       <c r="K19" t="s">
+        <v>166</v>
+      </c>
+      <c r="L19" t="s">
         <v>167</v>
-      </c>
-      <c r="L19" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
+        <v>168</v>
+      </c>
+      <c r="B20" t="s">
         <v>169</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>170</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>171</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>172</v>
-      </c>
-      <c r="E20" t="s">
-        <v>173</v>
       </c>
       <c r="F20" t="s">
         <v>39</v>
@@ -1418,36 +1406,36 @@
         <v>18</v>
       </c>
       <c r="H20" t="s">
+        <v>173</v>
+      </c>
+      <c r="I20" t="s">
+        <v>20</v>
+      </c>
+      <c r="J20" t="s">
         <v>174</v>
       </c>
-      <c r="I20" t="s">
-        <v>20</v>
-      </c>
-      <c r="J20" t="s">
+      <c r="K20" t="s">
+        <v>22</v>
+      </c>
+      <c r="L20" t="s">
         <v>175</v>
-      </c>
-      <c r="K20" t="s">
-        <v>176</v>
-      </c>
-      <c r="L20" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
+        <v>176</v>
+      </c>
+      <c r="B21" t="s">
+        <v>177</v>
+      </c>
+      <c r="C21" t="s">
         <v>178</v>
       </c>
-      <c r="B21" t="s">
+      <c r="D21" t="s">
         <v>179</v>
       </c>
-      <c r="C21" t="s">
+      <c r="E21" t="s">
         <v>180</v>
-      </c>
-      <c r="D21" t="s">
-        <v>181</v>
-      </c>
-      <c r="E21" t="s">
-        <v>182</v>
       </c>
       <c r="F21" t="s">
         <v>49</v>
@@ -1456,36 +1444,36 @@
         <v>18</v>
       </c>
       <c r="H21" t="s">
+        <v>181</v>
+      </c>
+      <c r="I21" t="s">
+        <v>20</v>
+      </c>
+      <c r="J21" t="s">
+        <v>182</v>
+      </c>
+      <c r="K21" t="s">
         <v>183</v>
       </c>
-      <c r="I21" t="s">
-        <v>20</v>
-      </c>
-      <c r="J21" t="s">
+      <c r="L21" t="s">
         <v>184</v>
-      </c>
-      <c r="K21" t="s">
-        <v>185</v>
-      </c>
-      <c r="L21" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
+        <v>185</v>
+      </c>
+      <c r="B22" t="s">
+        <v>186</v>
+      </c>
+      <c r="C22" t="s">
         <v>187</v>
       </c>
-      <c r="B22" t="s">
+      <c r="D22" t="s">
         <v>188</v>
       </c>
-      <c r="C22" t="s">
+      <c r="E22" t="s">
         <v>189</v>
-      </c>
-      <c r="D22" t="s">
-        <v>190</v>
-      </c>
-      <c r="E22" t="s">
-        <v>191</v>
       </c>
       <c r="F22" t="s">
         <v>17</v>
@@ -1494,7 +1482,7 @@
         <v>18</v>
       </c>
       <c r="H22" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="I22" t="s">
         <v>20</v>
@@ -1503,27 +1491,27 @@
         <v>31</v>
       </c>
       <c r="K22" t="s">
-        <v>193</v>
+        <v>95</v>
       </c>
       <c r="L22" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
+        <v>192</v>
+      </c>
+      <c r="B23" t="s">
+        <v>193</v>
+      </c>
+      <c r="C23" t="s">
+        <v>194</v>
+      </c>
+      <c r="D23" t="s">
         <v>195</v>
       </c>
-      <c r="B23" t="s">
+      <c r="E23" t="s">
         <v>196</v>
-      </c>
-      <c r="C23" t="s">
-        <v>197</v>
-      </c>
-      <c r="D23" t="s">
-        <v>198</v>
-      </c>
-      <c r="E23" t="s">
-        <v>199</v>
       </c>
       <c r="F23" t="s">
         <v>29</v>
@@ -1532,7 +1520,7 @@
         <v>50</v>
       </c>
       <c r="H23" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="I23" t="s">
         <v>20</v>
@@ -1541,27 +1529,27 @@
         <v>41</v>
       </c>
       <c r="K23" t="s">
-        <v>201</v>
+        <v>53</v>
       </c>
       <c r="L23" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
+        <v>199</v>
+      </c>
+      <c r="B24" t="s">
+        <v>200</v>
+      </c>
+      <c r="C24" t="s">
+        <v>201</v>
+      </c>
+      <c r="D24" t="s">
+        <v>202</v>
+      </c>
+      <c r="E24" t="s">
         <v>203</v>
-      </c>
-      <c r="B24" t="s">
-        <v>204</v>
-      </c>
-      <c r="C24" t="s">
-        <v>205</v>
-      </c>
-      <c r="D24" t="s">
-        <v>206</v>
-      </c>
-      <c r="E24" t="s">
-        <v>207</v>
       </c>
       <c r="F24" t="s">
         <v>39</v>
@@ -1570,7 +1558,7 @@
         <v>18</v>
       </c>
       <c r="H24" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="I24" t="s">
         <v>20</v>
@@ -1579,27 +1567,27 @@
         <v>52</v>
       </c>
       <c r="K24" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="L24" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
+        <v>207</v>
+      </c>
+      <c r="B25" t="s">
+        <v>208</v>
+      </c>
+      <c r="C25" t="s">
+        <v>209</v>
+      </c>
+      <c r="D25" t="s">
+        <v>210</v>
+      </c>
+      <c r="E25" t="s">
         <v>211</v>
-      </c>
-      <c r="B25" t="s">
-        <v>212</v>
-      </c>
-      <c r="C25" t="s">
-        <v>213</v>
-      </c>
-      <c r="D25" t="s">
-        <v>214</v>
-      </c>
-      <c r="E25" t="s">
-        <v>215</v>
       </c>
       <c r="F25" t="s">
         <v>49</v>
@@ -1608,7 +1596,7 @@
         <v>18</v>
       </c>
       <c r="H25" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="I25" t="s">
         <v>20</v>
@@ -1617,10 +1605,10 @@
         <v>61</v>
       </c>
       <c r="K25" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="L25" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>